<commit_message>
Scénario 3 : Test 1
Tester l’apport à 0% d’urine
</commit_message>
<xml_diff>
--- a/fiche_infos.xlsx
+++ b/fiche_infos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antoi\Documents\Cours ING5 S9\PFE\PyADM1-master\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6662443C-75E4-4ECD-9FA9-3698F807AF2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC79115-F94B-460E-93D8-AE92C37E6929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{08AD1386-BEB7-49B4-97A3-2BEA320D0E99}"/>
   </bookViews>
@@ -554,16 +554,16 @@
         <v>5</v>
       </c>
       <c r="L5" s="2">
+        <v>9</v>
+      </c>
+      <c r="M5" s="2">
         <v>6</v>
       </c>
-      <c r="M5" s="2">
+      <c r="N5" s="2">
         <v>7</v>
       </c>
-      <c r="N5" s="2">
+      <c r="O5" s="2">
         <v>8</v>
-      </c>
-      <c r="O5" s="2">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="5:16" x14ac:dyDescent="0.3">

</xml_diff>